<commit_message>
Added column "Database_number" to Datasets to available toggling afterwards
</commit_message>
<xml_diff>
--- a/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/MDPI_Parsed.xlsx
+++ b/Abschlussarbeit Bearbeitung/Jupyter Notebooks/1_Data-Acquisition-Wrapper/Gesammelte_Datenbanken/MDPI_Parsed.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\lucca\OneDrive\SPEICHER\Hochschule\7. Semester\Abschlussarbeit Bearbeitung\Jupyter Notebooks\1_Data-Acquisition-Wrapper\Gesammelte_Datenbanken\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99BF12B2-20F6-48D1-B107-C76BC0C3A61D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A721E8B4-30D5-4447-A445-BE6640DA1A54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="95">
   <si>
     <t>No</t>
   </si>
@@ -302,6 +302,9 @@
   </si>
   <si>
     <t>Southeast Tibet Plateau</t>
+  </si>
+  <si>
+    <t>Database_number</t>
   </si>
 </sst>
 </file>
@@ -701,14 +704,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AS53"/>
+  <dimension ref="A1:AT53"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="32.7109375" customWidth="1"/>
     <col min="20" max="20" width="16.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:45" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>92</v>
       </c>
@@ -844,8 +847,11 @@
       <c r="AS1" s="1" t="s">
         <v>91</v>
       </c>
-    </row>
-    <row r="2" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT1" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="2" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>93</v>
       </c>
@@ -909,8 +915,11 @@
       <c r="U2">
         <v>0.70871799999999996</v>
       </c>
-    </row>
-    <row r="3" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>93</v>
       </c>
@@ -974,8 +983,11 @@
       <c r="U3">
         <v>0.70871799999999996</v>
       </c>
-    </row>
-    <row r="4" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>93</v>
       </c>
@@ -1039,8 +1051,11 @@
       <c r="U4">
         <v>0.70871799999999996</v>
       </c>
-    </row>
-    <row r="5" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT4">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>93</v>
       </c>
@@ -1176,8 +1191,11 @@
       <c r="AS5">
         <v>2.0299999999999998</v>
       </c>
-    </row>
-    <row r="6" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT5">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>93</v>
       </c>
@@ -1241,8 +1259,11 @@
       <c r="U6">
         <v>0.70871799999999996</v>
       </c>
-    </row>
-    <row r="7" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT6">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>93</v>
       </c>
@@ -1303,8 +1324,11 @@
       <c r="U7">
         <v>0.70871799999999996</v>
       </c>
-    </row>
-    <row r="8" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>93</v>
       </c>
@@ -1368,8 +1392,11 @@
       <c r="U8">
         <v>0.70871799999999996</v>
       </c>
-    </row>
-    <row r="9" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT8">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>93</v>
       </c>
@@ -1433,8 +1460,11 @@
       <c r="U9">
         <v>0.70871799999999996</v>
       </c>
-    </row>
-    <row r="10" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>93</v>
       </c>
@@ -1498,8 +1528,11 @@
       <c r="U10">
         <v>0.70871799999999996</v>
       </c>
-    </row>
-    <row r="11" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT10">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>93</v>
       </c>
@@ -1563,8 +1596,11 @@
       <c r="U11">
         <v>0.70871799999999996</v>
       </c>
-    </row>
-    <row r="12" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT11">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>93</v>
       </c>
@@ -1697,8 +1733,11 @@
       <c r="AS12">
         <v>14.6</v>
       </c>
-    </row>
-    <row r="13" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>93</v>
       </c>
@@ -1762,8 +1801,11 @@
       <c r="U13">
         <v>0.71245499999999995</v>
       </c>
-    </row>
-    <row r="14" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>93</v>
       </c>
@@ -1827,8 +1869,11 @@
       <c r="U14">
         <v>0.71245499999999995</v>
       </c>
-    </row>
-    <row r="15" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT14">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="15" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>93</v>
       </c>
@@ -1892,8 +1937,11 @@
       <c r="U15">
         <v>0.71245499999999995</v>
       </c>
-    </row>
-    <row r="16" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT15">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="16" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>93</v>
       </c>
@@ -2029,8 +2077,11 @@
       <c r="AS16">
         <v>42.3</v>
       </c>
-    </row>
-    <row r="17" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT16">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="17" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>93</v>
       </c>
@@ -2088,8 +2139,11 @@
       <c r="U17">
         <v>0.70888700000000004</v>
       </c>
-    </row>
-    <row r="18" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT17">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>93</v>
       </c>
@@ -2153,8 +2207,11 @@
       <c r="U18">
         <v>0.70888700000000004</v>
       </c>
-    </row>
-    <row r="19" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT18">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="19" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>93</v>
       </c>
@@ -2218,8 +2275,11 @@
       <c r="U19">
         <v>0.70888700000000004</v>
       </c>
-    </row>
-    <row r="20" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT19">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>93</v>
       </c>
@@ -2283,8 +2343,11 @@
       <c r="U20">
         <v>0.70888700000000004</v>
       </c>
-    </row>
-    <row r="21" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT20">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="21" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>93</v>
       </c>
@@ -2348,8 +2411,11 @@
       <c r="U21">
         <v>0.70888700000000004</v>
       </c>
-    </row>
-    <row r="22" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT21">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>93</v>
       </c>
@@ -2413,8 +2479,11 @@
       <c r="U22">
         <v>0.70888700000000004</v>
       </c>
-    </row>
-    <row r="23" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT22">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>93</v>
       </c>
@@ -2550,8 +2619,11 @@
       <c r="AS23">
         <v>10.9</v>
       </c>
-    </row>
-    <row r="24" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT23">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="24" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>93</v>
       </c>
@@ -2612,8 +2684,11 @@
       <c r="U24">
         <v>0.70799800000000002</v>
       </c>
-    </row>
-    <row r="25" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT24">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>93</v>
       </c>
@@ -2677,8 +2752,11 @@
       <c r="U25">
         <v>0.70799800000000002</v>
       </c>
-    </row>
-    <row r="26" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>93</v>
       </c>
@@ -2742,8 +2820,11 @@
       <c r="U26">
         <v>0.70799800000000002</v>
       </c>
-    </row>
-    <row r="27" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT26">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>93</v>
       </c>
@@ -2807,8 +2888,11 @@
       <c r="U27">
         <v>0.70799800000000002</v>
       </c>
-    </row>
-    <row r="28" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT27">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>93</v>
       </c>
@@ -2944,8 +3028,11 @@
       <c r="AS28">
         <v>5.71</v>
       </c>
-    </row>
-    <row r="29" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT28">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>93</v>
       </c>
@@ -3009,8 +3096,11 @@
       <c r="U29">
         <v>0.71519900000000003</v>
       </c>
-    </row>
-    <row r="30" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT29">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="30" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>93</v>
       </c>
@@ -3074,8 +3164,11 @@
       <c r="U30">
         <v>0.71519900000000003</v>
       </c>
-    </row>
-    <row r="31" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT30">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>93</v>
       </c>
@@ -3139,8 +3232,11 @@
       <c r="U31">
         <v>0.71519900000000003</v>
       </c>
-    </row>
-    <row r="32" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT31">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>93</v>
       </c>
@@ -3204,8 +3300,11 @@
       <c r="U32">
         <v>0.71519900000000003</v>
       </c>
-    </row>
-    <row r="33" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT32">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="33" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>93</v>
       </c>
@@ -3269,8 +3368,11 @@
       <c r="U33">
         <v>0.71519900000000003</v>
       </c>
-    </row>
-    <row r="34" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT33">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>93</v>
       </c>
@@ -3406,8 +3508,11 @@
       <c r="AS34">
         <v>6.09</v>
       </c>
-    </row>
-    <row r="35" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT34">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>93</v>
       </c>
@@ -3468,8 +3573,11 @@
       <c r="U35">
         <v>0.71537399999999995</v>
       </c>
-    </row>
-    <row r="36" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>93</v>
       </c>
@@ -3533,8 +3641,11 @@
       <c r="U36">
         <v>0.71537399999999995</v>
       </c>
-    </row>
-    <row r="37" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT36">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>93</v>
       </c>
@@ -3598,8 +3709,11 @@
       <c r="U37">
         <v>0.71537399999999995</v>
       </c>
-    </row>
-    <row r="38" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>93</v>
       </c>
@@ -3663,8 +3777,11 @@
       <c r="U38">
         <v>0.71537399999999995</v>
       </c>
-    </row>
-    <row r="39" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>93</v>
       </c>
@@ -3728,8 +3845,11 @@
       <c r="U39">
         <v>0.71537399999999995</v>
       </c>
-    </row>
-    <row r="40" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>93</v>
       </c>
@@ -3865,8 +3985,11 @@
       <c r="AS40">
         <v>6.47</v>
       </c>
-    </row>
-    <row r="41" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT40">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>93</v>
       </c>
@@ -3930,8 +4053,11 @@
       <c r="U41">
         <v>0.71537399999999995</v>
       </c>
-    </row>
-    <row r="42" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>93</v>
       </c>
@@ -3995,8 +4121,11 @@
       <c r="U42">
         <v>0.71842600000000001</v>
       </c>
-    </row>
-    <row r="43" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT42">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>93</v>
       </c>
@@ -4045,8 +4174,11 @@
       <c r="U43">
         <v>0.71842600000000001</v>
       </c>
-    </row>
-    <row r="44" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT43">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>93</v>
       </c>
@@ -4095,8 +4227,11 @@
       <c r="U44">
         <v>0.71842600000000001</v>
       </c>
-    </row>
-    <row r="45" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT44">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="45" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>93</v>
       </c>
@@ -4145,8 +4280,11 @@
       <c r="U45">
         <v>0.71842600000000001</v>
       </c>
-    </row>
-    <row r="46" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT45">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>93</v>
       </c>
@@ -4282,8 +4420,11 @@
       <c r="AS46">
         <v>13.1</v>
       </c>
-    </row>
-    <row r="47" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT46">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="47" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>93</v>
       </c>
@@ -4344,8 +4485,11 @@
       <c r="U47">
         <v>0.71176099999999998</v>
       </c>
-    </row>
-    <row r="48" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT47">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="48" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>93</v>
       </c>
@@ -4406,8 +4550,11 @@
       <c r="U48">
         <v>0.71176099999999998</v>
       </c>
-    </row>
-    <row r="49" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT48">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="49" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>93</v>
       </c>
@@ -4471,8 +4618,11 @@
       <c r="U49">
         <v>0.71176099999999998</v>
       </c>
-    </row>
-    <row r="50" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT49">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="50" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>93</v>
       </c>
@@ -4536,8 +4686,11 @@
       <c r="U50">
         <v>0.71176099999999998</v>
       </c>
-    </row>
-    <row r="51" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT50">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="51" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>93</v>
       </c>
@@ -4601,8 +4754,11 @@
       <c r="U51">
         <v>0.71176099999999998</v>
       </c>
-    </row>
-    <row r="52" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT51">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="52" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>93</v>
       </c>
@@ -4738,8 +4894,11 @@
       <c r="AS52">
         <v>6.08</v>
       </c>
-    </row>
-    <row r="53" spans="1:45" x14ac:dyDescent="0.25">
+      <c r="AT52">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="53" spans="1:46" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>93</v>
       </c>
@@ -4859,6 +5018,9 @@
       </c>
       <c r="AS53">
         <v>36.9</v>
+      </c>
+      <c r="AT53">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>